<commit_message>
decompression_bfp8: fix test bench axis write issue
</commit_message>
<xml_diff>
--- a/library/decompression/bfp8.xlsx
+++ b/library/decompression/bfp8.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kele\Workspaces\hdl\library\decompression\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\hdl\library\decompression\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A726B5-056B-4718-B2EB-7AB4F1DA3D99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F500C9-1B8E-4AEF-9AFE-6A56BC0736DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="1080" windowWidth="21600" windowHeight="11295" xr2:uid="{CB36E99F-661D-4835-81D7-DB1D87AA1EF4}"/>
+    <workbookView xWindow="1260" yWindow="3405" windowWidth="22200" windowHeight="12180" xr2:uid="{CB36E99F-661D-4835-81D7-DB1D87AA1EF4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -194,13 +194,13 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -566,13 +566,13 @@
       <c r="C4" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="2" t="s">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="2" t="s">
         <v>1</v>
       </c>
       <c r="G4" s="3" t="s">
@@ -581,7 +581,7 @@
       <c r="H4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="J4" s="2" t="s">
@@ -619,7 +619,7 @@
       <c r="B5" s="9">
         <v>1</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="2" t="s">
@@ -643,27 +643,27 @@
       <c r="J5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="L5" s="12">
-        <v>1</v>
-      </c>
-      <c r="M5" s="12">
-        <v>1</v>
-      </c>
-      <c r="N5" s="12">
-        <v>1</v>
+      <c r="L5" s="14">
+        <v>1</v>
+      </c>
+      <c r="M5" s="14">
+        <v>1</v>
+      </c>
+      <c r="N5" s="14">
+        <v>0</v>
       </c>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
-      <c r="T5" s="2" t="s">
+      <c r="T5" s="5" t="s">
         <v>1</v>
       </c>
       <c r="U5" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="V5" s="2" t="s">
+      <c r="V5" s="5" t="s">
         <v>1</v>
       </c>
     </row>
@@ -695,10 +695,10 @@
       <c r="J6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
-      <c r="N6" s="12"/>
-      <c r="O6" s="6" t="s">
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="3" t="s">
         <v>2</v>
       </c>
       <c r="P6" s="1"/>
@@ -747,13 +747,13 @@
         <v>0</v>
       </c>
       <c r="O7" s="1"/>
-      <c r="P7" s="2" t="s">
+      <c r="P7" s="5" t="s">
         <v>1</v>
       </c>
       <c r="Q7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="R7" s="2" t="s">
+      <c r="R7" s="5" t="s">
         <v>1</v>
       </c>
       <c r="S7" s="3" t="s">
@@ -791,27 +791,27 @@
       <c r="J8" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L8" s="12">
+      <c r="L8" s="14">
         <v>3</v>
       </c>
-      <c r="M8" s="12">
-        <v>1</v>
-      </c>
-      <c r="N8" s="12">
-        <v>1</v>
+      <c r="M8" s="14">
+        <v>1</v>
+      </c>
+      <c r="N8" s="14">
+        <v>0</v>
       </c>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
-      <c r="T8" s="2" t="s">
+      <c r="T8" s="5" t="s">
         <v>1</v>
       </c>
       <c r="U8" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="V8" s="2" t="s">
+      <c r="V8" s="5" t="s">
         <v>1</v>
       </c>
     </row>
@@ -843,9 +843,9 @@
       <c r="J9" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L9" s="12"/>
-      <c r="M9" s="12"/>
-      <c r="N9" s="12"/>
+      <c r="L9" s="14"/>
+      <c r="M9" s="14"/>
+      <c r="N9" s="14"/>
       <c r="O9" s="3" t="s">
         <v>2</v>
       </c>
@@ -895,13 +895,13 @@
         <v>0</v>
       </c>
       <c r="O10" s="1"/>
-      <c r="P10" s="2" t="s">
+      <c r="P10" s="5" t="s">
         <v>1</v>
       </c>
       <c r="Q10" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="R10" s="2" t="s">
+      <c r="R10" s="5" t="s">
         <v>1</v>
       </c>
       <c r="S10" s="3" t="s">
@@ -939,27 +939,27 @@
       <c r="J11" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="L11" s="12">
+      <c r="L11" s="14">
         <v>5</v>
       </c>
-      <c r="M11" s="12">
-        <v>1</v>
-      </c>
-      <c r="N11" s="12">
-        <v>1</v>
+      <c r="M11" s="14">
+        <v>1</v>
+      </c>
+      <c r="N11" s="14">
+        <v>0</v>
       </c>
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
       <c r="S11" s="1"/>
-      <c r="T11" s="2" t="s">
+      <c r="T11" s="5" t="s">
         <v>1</v>
       </c>
       <c r="U11" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="V11" s="2" t="s">
+      <c r="V11" s="5" t="s">
         <v>1</v>
       </c>
     </row>
@@ -991,9 +991,9 @@
       <c r="J12" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="L12" s="12"/>
-      <c r="M12" s="12"/>
-      <c r="N12" s="12"/>
+      <c r="L12" s="14"/>
+      <c r="M12" s="14"/>
+      <c r="N12" s="14"/>
       <c r="O12" s="3" t="s">
         <v>2</v>
       </c>
@@ -1089,14 +1089,14 @@
       <c r="J14" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L14" s="12">
+      <c r="L14" s="14">
         <v>7</v>
       </c>
-      <c r="M14" s="12">
-        <v>1</v>
-      </c>
-      <c r="N14" s="12">
-        <v>1</v>
+      <c r="M14" s="14">
+        <v>1</v>
+      </c>
+      <c r="N14" s="14">
+        <v>0</v>
       </c>
       <c r="O14" s="1"/>
       <c r="P14" s="1"/>
@@ -1104,7 +1104,7 @@
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
       <c r="T14" s="1"/>
-      <c r="U14" s="2" t="s">
+      <c r="U14" s="5" t="s">
         <v>1</v>
       </c>
       <c r="V14" s="6" t="s">
@@ -1139,10 +1139,10 @@
       <c r="J15" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L15" s="12"/>
-      <c r="M15" s="12"/>
-      <c r="N15" s="12"/>
-      <c r="O15" s="2" t="s">
+      <c r="L15" s="14"/>
+      <c r="M15" s="14"/>
+      <c r="N15" s="14"/>
+      <c r="O15" s="5" t="s">
         <v>1</v>
       </c>
       <c r="P15" s="3" t="s">
@@ -1237,14 +1237,14 @@
       <c r="J17" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="L17" s="12">
+      <c r="L17" s="14">
         <v>9</v>
       </c>
-      <c r="M17" s="12">
-        <v>1</v>
-      </c>
-      <c r="N17" s="12">
-        <v>1</v>
+      <c r="M17" s="14">
+        <v>1</v>
+      </c>
+      <c r="N17" s="14">
+        <v>0</v>
       </c>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
@@ -1252,7 +1252,7 @@
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
-      <c r="U17" s="2" t="s">
+      <c r="U17" s="5" t="s">
         <v>1</v>
       </c>
       <c r="V17" s="6" t="s">
@@ -1287,10 +1287,10 @@
       <c r="J18" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="L18" s="12"/>
-      <c r="M18" s="12"/>
-      <c r="N18" s="12"/>
-      <c r="O18" s="2" t="s">
+      <c r="L18" s="14"/>
+      <c r="M18" s="14"/>
+      <c r="N18" s="14"/>
+      <c r="O18" s="5" t="s">
         <v>1</v>
       </c>
       <c r="P18" s="3" t="s">
@@ -1385,14 +1385,14 @@
       <c r="J20" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L20" s="12">
+      <c r="L20" s="14">
         <v>11</v>
       </c>
-      <c r="M20" s="12">
-        <v>1</v>
-      </c>
-      <c r="N20" s="12">
-        <v>1</v>
+      <c r="M20" s="14">
+        <v>1</v>
+      </c>
+      <c r="N20" s="14">
+        <v>0</v>
       </c>
       <c r="O20" s="1"/>
       <c r="P20" s="1"/>
@@ -1400,7 +1400,7 @@
       <c r="R20" s="1"/>
       <c r="S20" s="1"/>
       <c r="T20" s="1"/>
-      <c r="U20" s="2" t="s">
+      <c r="U20" s="5" t="s">
         <v>1</v>
       </c>
       <c r="V20" s="6" t="s">
@@ -1435,10 +1435,10 @@
       <c r="J21" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L21" s="12"/>
-      <c r="M21" s="12"/>
-      <c r="N21" s="12"/>
-      <c r="O21" s="2" t="s">
+      <c r="L21" s="14"/>
+      <c r="M21" s="14"/>
+      <c r="N21" s="14"/>
+      <c r="O21" s="5" t="s">
         <v>1</v>
       </c>
       <c r="P21" s="3" t="s">
@@ -1535,14 +1535,14 @@
       <c r="J23" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="L23" s="13">
+      <c r="L23" s="12">
         <v>13</v>
       </c>
-      <c r="M23" s="13">
-        <v>1</v>
-      </c>
-      <c r="N23" s="13">
-        <v>1</v>
+      <c r="M23" s="12">
+        <v>1</v>
+      </c>
+      <c r="N23" s="12">
+        <v>0</v>
       </c>
       <c r="O23" s="1"/>
       <c r="P23" s="1"/>
@@ -1551,7 +1551,7 @@
       <c r="S23" s="1"/>
       <c r="T23" s="1"/>
       <c r="U23" s="1"/>
-      <c r="V23" s="2" t="s">
+      <c r="V23" s="5" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1583,9 +1583,9 @@
       <c r="J24" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
-      <c r="N24" s="14"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="13"/>
+      <c r="N24" s="13"/>
       <c r="O24" s="3" t="s">
         <v>2</v>
       </c>
@@ -1683,14 +1683,14 @@
       <c r="J26" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L26" s="13">
+      <c r="L26" s="12">
         <v>15</v>
       </c>
-      <c r="M26" s="13">
-        <v>1</v>
-      </c>
-      <c r="N26" s="13">
-        <v>1</v>
+      <c r="M26" s="12">
+        <v>1</v>
+      </c>
+      <c r="N26" s="12">
+        <v>0</v>
       </c>
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
@@ -1699,7 +1699,7 @@
       <c r="S26" s="1"/>
       <c r="T26" s="1"/>
       <c r="U26" s="1"/>
-      <c r="V26" s="2" t="s">
+      <c r="V26" s="5" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1731,9 +1731,9 @@
       <c r="J27" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L27" s="14"/>
-      <c r="M27" s="14"/>
-      <c r="N27" s="14"/>
+      <c r="L27" s="13"/>
+      <c r="M27" s="13"/>
+      <c r="N27" s="13"/>
       <c r="O27" s="3" t="s">
         <v>2</v>
       </c>
@@ -1804,14 +1804,14 @@
       <c r="V28" s="1"/>
     </row>
     <row r="29" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="L29" s="13">
+      <c r="L29" s="12">
         <v>17</v>
       </c>
-      <c r="M29" s="13">
-        <v>1</v>
-      </c>
-      <c r="N29" s="13">
-        <v>1</v>
+      <c r="M29" s="12">
+        <v>1</v>
+      </c>
+      <c r="N29" s="12">
+        <v>0</v>
       </c>
       <c r="O29" s="1"/>
       <c r="P29" s="1"/>
@@ -1820,14 +1820,14 @@
       <c r="S29" s="1"/>
       <c r="T29" s="1"/>
       <c r="U29" s="1"/>
-      <c r="V29" s="2" t="s">
+      <c r="V29" s="5" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="L30" s="14"/>
-      <c r="M30" s="14"/>
-      <c r="N30" s="14"/>
+      <c r="L30" s="13"/>
+      <c r="M30" s="13"/>
+      <c r="N30" s="13"/>
       <c r="O30" s="3" t="s">
         <v>2</v>
       </c>
@@ -1880,7 +1880,7 @@
         <v>1</v>
       </c>
       <c r="N32" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O32" s="5" t="s">
         <v>1</v>
@@ -1934,7 +1934,7 @@
         <v>1</v>
       </c>
       <c r="N34" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O34" s="5" t="s">
         <v>1</v>
@@ -2008,14 +2008,14 @@
       <c r="V36" s="1"/>
     </row>
     <row r="37" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L37" s="13">
+      <c r="L37" s="12">
         <v>24</v>
       </c>
-      <c r="M37" s="13">
-        <v>1</v>
-      </c>
-      <c r="N37" s="13">
-        <v>1</v>
+      <c r="M37" s="12">
+        <v>1</v>
+      </c>
+      <c r="N37" s="12">
+        <v>0</v>
       </c>
       <c r="O37" s="1"/>
       <c r="P37" s="1"/>
@@ -2035,9 +2035,9 @@
       </c>
     </row>
     <row r="38" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L38" s="14"/>
-      <c r="M38" s="14"/>
-      <c r="N38" s="14"/>
+      <c r="L38" s="13"/>
+      <c r="M38" s="13"/>
+      <c r="N38" s="13"/>
       <c r="O38" s="3" t="s">
         <v>2</v>
       </c>
@@ -2077,14 +2077,14 @@
       <c r="V39" s="1"/>
     </row>
     <row r="40" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L40" s="13">
+      <c r="L40" s="12">
         <v>26</v>
       </c>
-      <c r="M40" s="13">
-        <v>1</v>
-      </c>
-      <c r="N40" s="13">
-        <v>1</v>
+      <c r="M40" s="12">
+        <v>1</v>
+      </c>
+      <c r="N40" s="12">
+        <v>0</v>
       </c>
       <c r="O40" s="1"/>
       <c r="P40" s="1"/>
@@ -2102,9 +2102,9 @@
       </c>
     </row>
     <row r="41" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L41" s="14"/>
-      <c r="M41" s="14"/>
-      <c r="N41" s="14"/>
+      <c r="L41" s="13"/>
+      <c r="M41" s="13"/>
+      <c r="N41" s="13"/>
       <c r="O41" s="3" t="s">
         <v>2</v>
       </c>
@@ -2144,13 +2144,13 @@
       <c r="V42" s="1"/>
     </row>
     <row r="43" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L43" s="13">
+      <c r="L43" s="12">
         <v>28</v>
       </c>
-      <c r="M43" s="13">
-        <v>1</v>
-      </c>
-      <c r="N43" s="13">
+      <c r="M43" s="12">
+        <v>1</v>
+      </c>
+      <c r="N43" s="12">
         <v>1</v>
       </c>
       <c r="O43" s="1"/>
@@ -2169,9 +2169,9 @@
       </c>
     </row>
     <row r="44" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L44" s="14"/>
-      <c r="M44" s="14"/>
-      <c r="N44" s="14"/>
+      <c r="L44" s="13"/>
+      <c r="M44" s="13"/>
+      <c r="N44" s="13"/>
       <c r="O44" s="3" t="s">
         <v>2</v>
       </c>
@@ -2211,14 +2211,14 @@
       <c r="V45" s="1"/>
     </row>
     <row r="46" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L46" s="13">
+      <c r="L46" s="12">
         <v>30</v>
       </c>
-      <c r="M46" s="13">
-        <v>1</v>
-      </c>
-      <c r="N46" s="13">
-        <v>1</v>
+      <c r="M46" s="12">
+        <v>1</v>
+      </c>
+      <c r="N46" s="12">
+        <v>0</v>
       </c>
       <c r="O46" s="1"/>
       <c r="P46" s="1"/>
@@ -2236,9 +2236,9 @@
       </c>
     </row>
     <row r="47" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L47" s="14"/>
-      <c r="M47" s="14"/>
-      <c r="N47" s="14"/>
+      <c r="L47" s="13"/>
+      <c r="M47" s="13"/>
+      <c r="N47" s="13"/>
       <c r="O47" s="5" t="s">
         <v>1</v>
       </c>
@@ -2280,14 +2280,14 @@
       <c r="V48" s="1"/>
     </row>
     <row r="49" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L49" s="13">
+      <c r="L49" s="12">
         <v>32</v>
       </c>
-      <c r="M49" s="13">
-        <v>1</v>
-      </c>
-      <c r="N49" s="13">
-        <v>1</v>
+      <c r="M49" s="12">
+        <v>1</v>
+      </c>
+      <c r="N49" s="12">
+        <v>0</v>
       </c>
       <c r="O49" s="1"/>
       <c r="P49" s="1"/>
@@ -2303,9 +2303,9 @@
       </c>
     </row>
     <row r="50" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L50" s="14"/>
-      <c r="M50" s="14"/>
-      <c r="N50" s="14"/>
+      <c r="L50" s="13"/>
+      <c r="M50" s="13"/>
+      <c r="N50" s="13"/>
       <c r="O50" s="5" t="s">
         <v>1</v>
       </c>
@@ -2347,13 +2347,13 @@
       <c r="V51" s="1"/>
     </row>
     <row r="52" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L52" s="13">
+      <c r="L52" s="12">
         <v>34</v>
       </c>
-      <c r="M52" s="13">
-        <v>1</v>
-      </c>
-      <c r="N52" s="13">
+      <c r="M52" s="12">
+        <v>1</v>
+      </c>
+      <c r="N52" s="12">
         <v>1</v>
       </c>
       <c r="O52" s="1"/>
@@ -2370,9 +2370,9 @@
       </c>
     </row>
     <row r="53" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L53" s="14"/>
-      <c r="M53" s="14"/>
-      <c r="N53" s="14"/>
+      <c r="L53" s="13"/>
+      <c r="M53" s="13"/>
+      <c r="N53" s="13"/>
       <c r="O53" s="5" t="s">
         <v>1</v>
       </c>
@@ -2414,14 +2414,14 @@
       <c r="V54" s="1"/>
     </row>
     <row r="55" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L55" s="13">
+      <c r="L55" s="12">
         <v>36</v>
       </c>
-      <c r="M55" s="13">
-        <v>1</v>
-      </c>
-      <c r="N55" s="13">
-        <v>1</v>
+      <c r="M55" s="12">
+        <v>1</v>
+      </c>
+      <c r="N55" s="12">
+        <v>0</v>
       </c>
       <c r="O55" s="1"/>
       <c r="P55" s="1"/>
@@ -2437,9 +2437,9 @@
       </c>
     </row>
     <row r="56" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L56" s="14"/>
-      <c r="M56" s="14"/>
-      <c r="N56" s="14"/>
+      <c r="L56" s="13"/>
+      <c r="M56" s="13"/>
+      <c r="N56" s="13"/>
       <c r="O56" s="3" t="s">
         <v>2</v>
       </c>
@@ -2483,14 +2483,14 @@
       <c r="V57" s="1"/>
     </row>
     <row r="58" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L58" s="13">
+      <c r="L58" s="12">
         <v>38</v>
       </c>
-      <c r="M58" s="13">
-        <v>1</v>
-      </c>
-      <c r="N58" s="13">
-        <v>1</v>
+      <c r="M58" s="12">
+        <v>1</v>
+      </c>
+      <c r="N58" s="12">
+        <v>0</v>
       </c>
       <c r="O58" s="1"/>
       <c r="P58" s="1"/>
@@ -2504,9 +2504,9 @@
       </c>
     </row>
     <row r="59" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L59" s="14"/>
-      <c r="M59" s="14"/>
-      <c r="N59" s="14"/>
+      <c r="L59" s="13"/>
+      <c r="M59" s="13"/>
+      <c r="N59" s="13"/>
       <c r="O59" s="3" t="s">
         <v>2</v>
       </c>
@@ -2550,13 +2550,13 @@
       <c r="V60" s="1"/>
     </row>
     <row r="61" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L61" s="13">
+      <c r="L61" s="12">
         <v>40</v>
       </c>
-      <c r="M61" s="13">
-        <v>1</v>
-      </c>
-      <c r="N61" s="13">
+      <c r="M61" s="12">
+        <v>1</v>
+      </c>
+      <c r="N61" s="12">
         <v>1</v>
       </c>
       <c r="O61" s="1"/>
@@ -2571,9 +2571,9 @@
       </c>
     </row>
     <row r="62" spans="12:22" x14ac:dyDescent="0.25">
-      <c r="L62" s="14"/>
-      <c r="M62" s="14"/>
-      <c r="N62" s="14"/>
+      <c r="L62" s="13"/>
+      <c r="M62" s="13"/>
+      <c r="N62" s="13"/>
       <c r="O62" s="3" t="s">
         <v>2</v>
       </c>
@@ -2626,7 +2626,7 @@
         <v>1</v>
       </c>
       <c r="N64" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O64" s="5" t="s">
         <v>1</v>
@@ -2680,7 +2680,7 @@
         <v>1</v>
       </c>
       <c r="N66" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O66" s="5" t="s">
         <v>1</v>
@@ -2787,36 +2787,24 @@
       </c>
       <c r="N70">
         <f>SUM(N4:N69)</f>
-        <v>23</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="N55:N56"/>
-    <mergeCell ref="N58:N59"/>
-    <mergeCell ref="N61:N62"/>
-    <mergeCell ref="N40:N41"/>
-    <mergeCell ref="N43:N44"/>
-    <mergeCell ref="N46:N47"/>
-    <mergeCell ref="N49:N50"/>
-    <mergeCell ref="N52:N53"/>
-    <mergeCell ref="N20:N21"/>
-    <mergeCell ref="N23:N24"/>
-    <mergeCell ref="N26:N27"/>
-    <mergeCell ref="N29:N30"/>
-    <mergeCell ref="N37:N38"/>
-    <mergeCell ref="N5:N6"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="N14:N15"/>
-    <mergeCell ref="N17:N18"/>
-    <mergeCell ref="L40:L41"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="L14:L15"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="L20:L21"/>
+    <mergeCell ref="M58:M59"/>
+    <mergeCell ref="M61:M62"/>
+    <mergeCell ref="M40:M41"/>
+    <mergeCell ref="M43:M44"/>
+    <mergeCell ref="M46:M47"/>
+    <mergeCell ref="M49:M50"/>
+    <mergeCell ref="M52:M53"/>
+    <mergeCell ref="M55:M56"/>
+    <mergeCell ref="M17:M18"/>
+    <mergeCell ref="M20:M21"/>
+    <mergeCell ref="M23:M24"/>
+    <mergeCell ref="M26:M27"/>
+    <mergeCell ref="M29:M30"/>
     <mergeCell ref="M37:M38"/>
     <mergeCell ref="L61:L62"/>
     <mergeCell ref="M5:M6"/>
@@ -2833,19 +2821,31 @@
     <mergeCell ref="L26:L27"/>
     <mergeCell ref="L29:L30"/>
     <mergeCell ref="L37:L38"/>
-    <mergeCell ref="M17:M18"/>
-    <mergeCell ref="M20:M21"/>
-    <mergeCell ref="M23:M24"/>
-    <mergeCell ref="M26:M27"/>
-    <mergeCell ref="M29:M30"/>
-    <mergeCell ref="M58:M59"/>
-    <mergeCell ref="M61:M62"/>
-    <mergeCell ref="M40:M41"/>
-    <mergeCell ref="M43:M44"/>
-    <mergeCell ref="M46:M47"/>
-    <mergeCell ref="M49:M50"/>
-    <mergeCell ref="M52:M53"/>
-    <mergeCell ref="M55:M56"/>
+    <mergeCell ref="L40:L41"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="L20:L21"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="N14:N15"/>
+    <mergeCell ref="N17:N18"/>
+    <mergeCell ref="N20:N21"/>
+    <mergeCell ref="N23:N24"/>
+    <mergeCell ref="N26:N27"/>
+    <mergeCell ref="N29:N30"/>
+    <mergeCell ref="N37:N38"/>
+    <mergeCell ref="N55:N56"/>
+    <mergeCell ref="N58:N59"/>
+    <mergeCell ref="N61:N62"/>
+    <mergeCell ref="N40:N41"/>
+    <mergeCell ref="N43:N44"/>
+    <mergeCell ref="N46:N47"/>
+    <mergeCell ref="N49:N50"/>
+    <mergeCell ref="N52:N53"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>